<commit_message>
GUI kodlu versiyon eklendi
</commit_message>
<xml_diff>
--- a/Test Sonuclari/TestSonuclari.xlsx
+++ b/Test Sonuclari/TestSonuclari.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW4"/>
+  <dimension ref="A1:AW6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -441,16 +441,16 @@
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="45" customWidth="1" min="19" max="19"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
     <col width="30" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="45" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
     <col width="45" customWidth="1" min="23" max="23"/>
     <col width="45" customWidth="1" min="24" max="24"/>
@@ -459,7 +459,7 @@
     <col width="45" customWidth="1" min="27" max="27"/>
     <col width="45" customWidth="1" min="28" max="28"/>
     <col width="45" customWidth="1" min="29" max="29"/>
-    <col width="45" customWidth="1" min="30" max="30"/>
+    <col width="40" customWidth="1" min="30" max="30"/>
     <col width="40" customWidth="1" min="31" max="31"/>
     <col width="40" customWidth="1" min="32" max="32"/>
     <col width="40" customWidth="1" min="33" max="33"/>
@@ -539,152 +539,152 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mag Kalib Yüklenmesi</t>
+          <t>Kalibrasyon - Config Kontrol Sonucu</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Kalibrasyon - Config Kontrol Sonucu</t>
+          <t>Hard Reset - 1 Sonucu:</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Hard Reset - 1 Sonucu:</t>
+          <t>Hard Reset - 2 Sonucu:</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Hard Reset - 2 Sonucu:</t>
+          <t>Soft Reset - 1 Sonucu:</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Soft Reset - 1 Sonucu:</t>
+          <t>Soft Reset - 2 Sonucu:</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Soft Reset - 2 Sonucu:</t>
+          <t>Reset Testi Sonucu:</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Reset Testi Sonucu:</t>
+          <t>Acc Norm Açılış Sonucu:</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Acc Norm Açılış Sonucu:</t>
+          <t>Max Acc Norm Değeri:</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Max Acc Norm Değeri:</t>
+          <t>Min Acc Norm Değeri:</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Min Acc Norm Değeri:</t>
+          <t>Acc Norm Status:</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Acc Norm Status:</t>
+          <t>Gyro Açılış Sonucu:</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Gyro Açılış Sonucu:</t>
+          <t>Acc Döndürme Test - 1 Sonucu:</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 1 Sonucu:</t>
+          <t>Acc Döndürme Test - 2 Sonucu:</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 2 Sonucu:</t>
+          <t>Acc Döndürme Test - 3 Sonucu:</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 3 Sonucu:</t>
+          <t>Acc Döndürme Test - 4 Sonucu:</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 4 Sonucu:</t>
+          <t>Acc Döndürme Test - 5 Sonucu:</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 5 Sonucu:</t>
+          <t>Acc Döndürme Test - 6 Sonucu:</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test - 6 Sonucu:</t>
+          <t>Acc Döndürme Test Sonucu:</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Acc Döndürme Test Sonucu:</t>
+          <t>Konum 1 Roll Ortalaması:</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Konum 1 Roll Ortalaması:</t>
+          <t>Konum 1 Pitch Ortalaması:</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Konum 1 Pitch Ortalaması:</t>
+          <t>Konum 2 Roll Ortalaması:</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Konum 2 Roll Ortalaması:</t>
+          <t>Konum 2 Pitch Ortalaması:</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Konum 2 Pitch Ortalaması:</t>
+          <t>Konum 3 Roll Ortalaması:</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Konum 3 Roll Ortalaması:</t>
+          <t>Konum 3 Pitch Ortalaması:</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>Konum 3 Pitch Ortalaması:</t>
+          <t>Euler Test Sonucu:</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>Euler Test Sonucu:</t>
+          <t>Gyro Z Testi Yaw Farkı:</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>Gyro Z Testi Yaw Farkı:</t>
+          <t>Gyro Z Test Sonucu:</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>Gyro Z Test Sonucu:</t>
+          <t>RS 232 Bağlantı Sonucu:</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>RS 232 Bağlantı Sonucu:</t>
+          <t>RS 422 Bağlantı Sonucu:</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>RS 422 Bağlantı Sonucu:</t>
+          <t>RS 232-422 Bağlantı Sonucu:</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
@@ -779,14 +779,19 @@
           <t>Yüklü Olmalı</t>
         </is>
       </c>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>9.82</t>
+        </is>
+      </c>
       <c r="T2" s="1" t="inlineStr">
         <is>
-          <t>9.82</t>
+          <t>9.78</t>
         </is>
       </c>
       <c r="U2" s="1" t="inlineStr">
         <is>
-          <t>9.78</t>
+          <t>Best veya Noted</t>
         </is>
       </c>
       <c r="V2" s="1" t="inlineStr">
@@ -794,6 +799,11 @@
           <t>Best veya Noted</t>
         </is>
       </c>
+      <c r="AD2" s="1" t="inlineStr">
+        <is>
+          <t>0.15'ten küçük olmalı:</t>
+        </is>
+      </c>
       <c r="AE2" s="1" t="inlineStr">
         <is>
           <t>0.15'ten küçük olmalı:</t>
@@ -801,27 +811,27 @@
       </c>
       <c r="AF2" s="1" t="inlineStr">
         <is>
+          <t>89.85 - 90 aralığında olmalı:</t>
+        </is>
+      </c>
+      <c r="AG2" s="1" t="inlineStr">
+        <is>
           <t>0.15'ten küçük olmalı:</t>
         </is>
       </c>
-      <c r="AG2" s="1" t="inlineStr">
-        <is>
-          <t>89.85 - 90 aralığında olmalı:</t>
-        </is>
-      </c>
       <c r="AH2" s="1" t="inlineStr">
         <is>
+          <t>179.85 - 180 aralığında olmalı:</t>
+        </is>
+      </c>
+      <c r="AI2" s="1" t="inlineStr">
+        <is>
           <t>0.15'ten küçük olmalı:</t>
         </is>
       </c>
-      <c r="AI2" s="1" t="inlineStr">
-        <is>
-          <t>179.85 - 180 aralığında olmalı:</t>
-        </is>
-      </c>
       <c r="AJ2" s="1" t="inlineStr">
         <is>
-          <t>0.15'ten küçük olmalı:</t>
+          <t>0.3'ten küçük olmalı:</t>
         </is>
       </c>
       <c r="AK2" s="1" t="inlineStr">
@@ -852,7 +862,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46297.47664075645</v>
+        <v>46297.47664075231</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
@@ -1058,7 +1068,365 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>25325220</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46301.54177081019</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SN Eşleşti</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FW Eşleşti</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>DN Eşleşti</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>HW Eşleşti</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Acc Kalib Yüklü</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Gyro Kalib Yüklü</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>9.787121378148397</v>
+      </c>
+      <c r="U4" t="n">
+        <v>9.787121378148397</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.5440277392967192</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>-0.5438781850456846</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.5441290786805101</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>-0.5533561066344436</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.5475784544402469</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>-0.5495018683445645</v>
+      </c>
+      <c r="AK4" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.1940045596629352</v>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>25325220</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46301.56388732705</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SN Eşleşti</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FW Eşleşti</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>DN Eşleşti</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>HW Eşleşti</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Acc Kalib Yüklü</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Gyro Kalib Yüklü</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>9.78903297512465</v>
+      </c>
+      <c r="U5" t="n">
+        <v>9.78903297512465</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="Z5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AB5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.5467747542937083</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>-0.5482196819863102</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0.5376591211436257</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>-0.5396669739070354</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0.5471154508384267</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>-0.5398845055337164</v>
+      </c>
+      <c r="AK5" s="3" t="inlineStr">
+        <is>
+          <t>Kaldı</t>
+        </is>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.09310062775509359</v>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Geçti</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>